<commit_message>
corpus(rs2): the wall's limit-equilibrium files stop declaring a K0
vp088 and vp090 carried the vendor's K0 = 1 in main!D16 for a strength-reduction
row that printed a number with no tag behind it, which is why the K0 guard kept
a two-name exception list. That row runs on vp088_fem and vp090_fem now, so the
two files no longer need an initial stress state at all: they are rebuilt
without one, the exception list is empty, and the rebuild guard reproduces all
154 targets where it reported a K0 difference on these two before.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/vp088.xlsx
+++ b/docs/verification/files/rocscience/vp088.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523500CF-89B8-4644-B955-31C74218CF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904BD95E-2C21-0841-A7DF-ECBA420EAAD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27680" yWindow="3200" windowWidth="31600" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="323">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t>vg</t>
-  </si>
-  <si>
-    <t>van Genuchten model (a, n)</t>
   </si>
   <si>
     <t>pow</t>
@@ -1134,6 +1131,24 @@
   </si>
   <si>
     <t>Unrotated</t>
+  </si>
+  <si>
+    <t>van Genuchten model (a, n, l)</t>
+  </si>
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>Joint</t>
+  </si>
+  <si>
+    <t>kn</t>
+  </si>
+  <si>
+    <t>ks</t>
+  </si>
+  <si>
+    <t>Jred</t>
   </si>
 </sst>
 </file>
@@ -1641,7 +1656,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="37">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1904,16 +1933,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>217714</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>54430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>29</xdr:col>
       <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>90714</xdr:rowOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>18143</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1928,8 +1957,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16455571" y="254001"/>
-          <a:ext cx="3855358" cy="4027713"/>
+          <a:off x="19757571" y="254001"/>
+          <a:ext cx="3855358" cy="4753428"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2102,7 +2131,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = residual capacity after rupture (FEM only)</a:t>
+            <a:t> = residual capacity after rupture</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2112,7 +2141,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = modulus of elasticity of reinforcement (FEM only)</a:t>
+            <a:t> = modulus of elasticity of reinforcement</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2122,7 +2151,48 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = cross-sectional area of reinforcement (FEM only)</a:t>
+            <a:t> = cross-sectional area of reinforcement</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Joint</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = model as slip element; mesh splits along line</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>kn</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint normal stiffness (blank = from soil E and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>ks</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint shear stiffness (blank = from soil G and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Jred</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = reduce joint strength in SSRM (blank = Yes)</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="en-US" sz="1100" b="0"/>
@@ -2881,7 +2951,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3016,9 +3086,7 @@
       <c r="G16" t="s">
         <v>34</v>
       </c>
-      <c r="D16">
-        <v>1.0</v>
-      </c>
+      <c r="D16"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
@@ -3059,7 +3127,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>46</v>
@@ -3154,7 +3222,7 @@
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D58" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.2">
@@ -3283,89 +3351,101 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A2:AD25"/>
+  <dimension ref="A2:AH29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="6" width="10.83203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" customWidth="1"/>
     <col min="10" max="14" width="10.83203125" style="1" customWidth="1"/>
-    <col min="18" max="20" width="10.83203125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="4.33203125" customWidth="1"/>
+    <col min="18" max="24" width="10.83203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="40" t="s">
         <v>246</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="H2" s="40" t="s">
         <v>247</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="I2" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="J2" s="27" t="s">
         <v>249</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="L2" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="M2" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="O2" s="27" t="s">
         <v>252</v>
       </c>
-      <c r="M2" s="27" t="s">
-        <v>311</v>
-      </c>
-      <c r="N2" s="27" t="s">
-        <v>312</v>
-      </c>
-      <c r="O2" s="27" t="s">
+      <c r="P2" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="P2" s="27" t="s">
+      <c r="Q2" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="Q2" s="27" t="s">
+      <c r="R2" s="28" t="s">
         <v>255</v>
       </c>
-      <c r="R2" s="28" t="s">
+      <c r="S2" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="T2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="S2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="T2" s="28" t="s">
+      <c r="U2" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="V2" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="W2" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="X2" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="AF2" t="s">
         <v>257</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AG2" t="s">
         <v>258</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AH2" t="s">
         <v>259</v>
       </c>
-      <c r="AD2" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3428,17 +3508,21 @@
       <c r="T3" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="AF3" t="s">
+        <v>260</v>
+      </c>
+      <c r="AG3" t="s">
         <v>261</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AH3" t="s">
         <v>262</v>
       </c>
-      <c r="AD3" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3501,11 +3585,15 @@
       <c r="T4" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB4" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="AF4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3568,11 +3656,15 @@
       <c r="T5" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB5" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="AF5" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3635,8 +3727,12 @@
       <c r="T6" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3699,8 +3795,12 @@
       <c r="T7" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3763,17 +3863,21 @@
       <c r="T8" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB8" t="s">
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="AF8" t="s">
+        <v>257</v>
+      </c>
+      <c r="AG8" t="s">
         <v>258</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AH8" t="s">
         <v>259</v>
       </c>
-      <c r="AD8" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3836,17 +3940,21 @@
       <c r="T9" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB9" t="s">
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="AF9" t="s">
+        <v>260</v>
+      </c>
+      <c r="AG9" t="s">
         <v>261</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AH9" t="s">
         <v>262</v>
       </c>
-      <c r="AD9" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3909,17 +4017,21 @@
       <c r="T10" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB10" t="s">
-        <v>264</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>262</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+      <c r="AF10" t="s">
+        <v>263</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>261</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3982,17 +4094,21 @@
       <c r="T11" s="3">
         <v>0.1</v>
       </c>
-      <c r="AB11" t="s">
-        <v>265</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>262</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+      <c r="AF11" t="s">
+        <v>264</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>261</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -4055,8 +4171,12 @@
       <c r="T12" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -4119,8 +4239,12 @@
       <c r="T13" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -4183,8 +4307,12 @@
       <c r="T14" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -4247,8 +4375,12 @@
       <c r="T15" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="3"/>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -4311,8 +4443,12 @@
       <c r="T16" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -4375,8 +4511,12 @@
       <c r="T17" s="3">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -4387,11 +4527,11 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="str">
-        <f>IF($G18="","",IFERROR(VLOOKUP($G18,$AB$8:$AD$11,2,0),""))</f>
+        <f>IF($G18="","",IFERROR(VLOOKUP($G18,$AF$8:$AH$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I18" s="3" t="str">
-        <f>IF($G18="","",IFERROR(VLOOKUP($G18,$AB$8:$AD$11,3,0),""))</f>
+        <f>IF($G18="","",IFERROR(VLOOKUP($G18,$AF$8:$AH$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J18" s="3"/>
@@ -4405,8 +4545,12 @@
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -4417,11 +4561,11 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3" t="str">
-        <f>IF($G19="","",IFERROR(VLOOKUP($G19,$AB$8:$AD$11,2,0),""))</f>
+        <f>IF($G19="","",IFERROR(VLOOKUP($G19,$AF$8:$AH$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I19" s="3" t="str">
-        <f>IF($G19="","",IFERROR(VLOOKUP($G19,$AB$8:$AD$11,3,0),""))</f>
+        <f>IF($G19="","",IFERROR(VLOOKUP($G19,$AF$8:$AH$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J19" s="3"/>
@@ -4435,8 +4579,12 @@
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -4447,11 +4595,11 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="str">
-        <f>IF($G20="","",IFERROR(VLOOKUP($G20,$AB$8:$AD$11,2,0),""))</f>
+        <f>IF($G20="","",IFERROR(VLOOKUP($G20,$AF$8:$AH$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I20" s="3" t="str">
-        <f>IF($G20="","",IFERROR(VLOOKUP($G20,$AB$8:$AD$11,3,0),""))</f>
+        <f>IF($G20="","",IFERROR(VLOOKUP($G20,$AF$8:$AH$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J20" s="3"/>
@@ -4465,8 +4613,12 @@
       <c r="R20" s="3"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
+      <c r="X20" s="3"/>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -4477,11 +4629,11 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="str">
-        <f>IF($G21="","",IFERROR(VLOOKUP($G21,$AB$8:$AD$11,2,0),""))</f>
+        <f>IF($G21="","",IFERROR(VLOOKUP($G21,$AF$8:$AH$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I21" s="3" t="str">
-        <f>IF($G21="","",IFERROR(VLOOKUP($G21,$AB$8:$AD$11,3,0),""))</f>
+        <f>IF($G21="","",IFERROR(VLOOKUP($G21,$AF$8:$AH$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J21" s="3"/>
@@ -4495,8 +4647,12 @@
       <c r="R21" s="3"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="3"/>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -4507,11 +4663,11 @@
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="str">
-        <f>IF($G22="","",IFERROR(VLOOKUP($G22,$AB$8:$AD$11,2,0),""))</f>
+        <f>IF($G22="","",IFERROR(VLOOKUP($G22,$AF$8:$AH$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I22" s="3" t="str">
-        <f>IF($G22="","",IFERROR(VLOOKUP($G22,$AB$8:$AD$11,3,0),""))</f>
+        <f>IF($G22="","",IFERROR(VLOOKUP($G22,$AF$8:$AH$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J22" s="3"/>
@@ -4525,39 +4681,60 @@
       <c r="R22" s="3"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="V23" s="42"/>
-      <c r="W23" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="V24" s="26"/>
-      <c r="W24" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="V25" s="29"/>
-      <c r="W25" s="9" t="s">
-        <v>104</v>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z27" s="42"/>
+      <c r="AA27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z28" s="26"/>
+      <c r="AA28" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z29" s="29"/>
+      <c r="AA29" s="9" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <conditionalFormatting sqref="K3:L22">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$U3="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V3:X22">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>$U3&lt;&gt;"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G22" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>$AB$2:$AB$5</formula1>
+      <formula1>$AF$2:$AF$5</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H22" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>$AC$2:$AC$3</formula1>
+      <formula1>$AG$2:$AG$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I22" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>$AD$2:$AD$3</formula1>
+      <formula1>$AH$2:$AH$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U3:U22 X3:X22" xr:uid="{8FB27197-C456-2D4D-8100-E78D5059F972}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4580,61 +4757,61 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>246</v>
-      </c>
       <c r="G2" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="I2" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="H2" s="40" t="s">
-        <v>249</v>
-      </c>
-      <c r="I2" s="27" t="s">
+      <c r="J2" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="41" t="s">
         <v>268</v>
       </c>
-      <c r="K2" s="41" t="s">
+      <c r="L2" s="41" t="s">
         <v>269</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="M2" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="N2" s="28" t="s">
         <v>270</v>
       </c>
-      <c r="M2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="N2" s="28" t="s">
-        <v>271</v>
-      </c>
       <c r="O2" s="28" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="P2" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q2" s="28" t="s">
         <v>314</v>
       </c>
-      <c r="Q2" s="28" t="s">
-        <v>315</v>
-      </c>
       <c r="Z2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AA2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -4658,10 +4835,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AA3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -4685,7 +4862,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="Z4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
@@ -4709,7 +4886,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="Z5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
@@ -4872,13 +5049,13 @@
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="S16" s="26"/>
       <c r="T16" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="19:20" x14ac:dyDescent="0.2">
       <c r="S17" s="29"/>
       <c r="T17" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4907,22 +5084,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>167</v>
-      </c>
       <c r="E2" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>272</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -5145,27 +5322,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -5173,71 +5350,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F3" s="33"/>
       <c r="H3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I3" s="33"/>
       <c r="K3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -5254,10 +5431,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="U5" t="s">
         <v>283</v>
-      </c>
-      <c r="U5" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -5274,7 +5451,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -5563,27 +5740,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -5591,71 +5768,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F3" s="35"/>
       <c r="H3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I3" s="35"/>
       <c r="K3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -5672,10 +5849,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="U5" t="s">
         <v>283</v>
-      </c>
-      <c r="U5" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -5974,22 +6151,22 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B2" s="50" t="s">
+        <v>291</v>
+      </c>
+      <c r="C2" s="50" t="s">
         <v>292</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="D2" s="50" t="s">
         <v>293</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="E2" s="50" t="s">
         <v>294</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>296</v>
-      </c>
-      <c r="G2" s="50" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
@@ -6000,7 +6177,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="I3" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -6022,7 +6199,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -6044,7 +6221,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -6056,7 +6233,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="I8" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -6068,7 +6245,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" s="14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -6088,7 +6265,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="J11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
@@ -6899,16 +7076,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:AP52"/>
+  <dimension ref="A2:AQ52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="41" width="8.5" customWidth="1"/>
+    <col min="11" max="42" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>79</v>
       </c>
@@ -6923,7 +7100,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>83</v>
       </c>
@@ -6944,7 +7121,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>89</v>
       </c>
@@ -6966,67 +7143,67 @@
         <v>93</v>
       </c>
       <c r="AK4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="C5" s="1" t="s">
+      <c r="D5" t="s">
         <v>95</v>
-      </c>
-      <c r="D5" t="s">
-        <v>96</v>
       </c>
       <c r="L5" s="26"/>
       <c r="M5" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="O5" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="P5" s="9" t="s">
         <v>98</v>
-      </c>
-      <c r="P5" s="9" t="s">
-        <v>99</v>
       </c>
       <c r="AD5" s="14"/>
       <c r="AJ5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AK5" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="AK5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="L6" s="29"/>
       <c r="M6" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="O6" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="P6" t="s">
         <v>105</v>
-      </c>
-      <c r="P6" t="s">
-        <v>106</v>
       </c>
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C9" s="53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="52"/>
@@ -7052,7 +7229,7 @@
       <c r="Y9" s="54"/>
       <c r="Z9" s="54"/>
       <c r="AA9" s="53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -7060,7 +7237,7 @@
       <c r="AE9" s="54"/>
       <c r="AF9" s="54"/>
       <c r="AG9" s="53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH9" s="54"/>
       <c r="AI9" s="54"/>
@@ -7071,136 +7248,140 @@
       <c r="AN9" s="54"/>
       <c r="AO9" s="54"/>
       <c r="AP9" s="54"/>
-    </row>
-    <row r="10" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AQ9" s="54"/>
+    </row>
+    <row r="10" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="45" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="D10" s="48" t="s">
+        <v>308</v>
+      </c>
+      <c r="E10" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="E10" s="44" t="s">
+      <c r="F10" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="G10" s="45" t="s">
         <v>115</v>
       </c>
-      <c r="G10" s="45" t="s">
+      <c r="H10" s="44" t="s">
         <v>116</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="I10" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="I10" s="44" t="s">
+      <c r="J10" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="J10" s="49" t="s">
+      <c r="K10" s="49" t="s">
         <v>119</v>
       </c>
-      <c r="K10" s="49" t="s">
+      <c r="L10" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="M10" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="N10" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="N10" s="43" t="s">
+      <c r="O10" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="O10" s="44" t="s">
+      <c r="P10" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="P10" s="44" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q10" s="44" t="s">
+      <c r="R10" s="44" t="s">
         <v>125</v>
       </c>
-      <c r="R10" s="44" t="s">
+      <c r="S10" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="S10" s="44" t="s">
+      <c r="T10" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="T10" s="44" t="s">
+      <c r="U10" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="U10" s="44" t="s">
+      <c r="V10" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="V10" s="44" t="s">
+      <c r="W10" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="W10" s="44" t="s">
+      <c r="X10" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="X10" s="44" t="s">
+      <c r="Y10" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="Y10" s="44" t="s">
+      <c r="Z10" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="Z10" s="44" t="s">
+      <c r="AA10" s="46" t="s">
+        <v>304</v>
+      </c>
+      <c r="AB10" s="46" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC10" s="47" t="s">
         <v>134</v>
       </c>
-      <c r="AA10" s="46" t="s">
+      <c r="AD10" s="46" t="s">
         <v>305</v>
       </c>
-      <c r="AB10" s="46" t="s">
-        <v>304</v>
-      </c>
-      <c r="AC10" s="47" t="s">
+      <c r="AE10" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="AF10" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="AG10" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="AD10" s="46" t="s">
-        <v>306</v>
-      </c>
-      <c r="AE10" s="46" t="s">
-        <v>307</v>
-      </c>
-      <c r="AF10" s="47" t="s">
-        <v>308</v>
-      </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AH10" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AI10" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AJ10" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AK10" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="AM10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AN10" s="23" t="s">
+      <c r="AO10" s="23" t="s">
+        <v>318</v>
+      </c>
+      <c r="AP10" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AO10" s="23" t="s">
+      <c r="AQ10" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="AP10" s="23" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -7323,10 +7504,13 @@
       <c r="AN11" s="3">
         <v>0.0</v>
       </c>
-      <c r="AO11" s="3"/>
+      <c r="AO11" s="3">
+        <v>0.5</v>
+      </c>
       <c r="AP11" s="3"/>
-    </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ11" s="3"/>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -7449,10 +7633,13 @@
       <c r="AN12" s="19">
         <v>0.0</v>
       </c>
-      <c r="AO12" s="19"/>
+      <c r="AO12" s="19">
+        <v>0.5</v>
+      </c>
       <c r="AP12" s="19"/>
-    </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ12" s="19"/>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -7575,10 +7762,13 @@
       <c r="AN13" s="19">
         <v>0.0</v>
       </c>
-      <c r="AO13" s="19"/>
+      <c r="AO13" s="19">
+        <v>0.5</v>
+      </c>
       <c r="AP13" s="19"/>
-    </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ13" s="19"/>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -7623,8 +7813,9 @@
       <c r="AN14" s="3"/>
       <c r="AO14" s="3"/>
       <c r="AP14" s="3"/>
-    </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ14" s="3"/>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -7669,8 +7860,9 @@
       <c r="AN15" s="3"/>
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
-    </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ15" s="3"/>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -7715,8 +7907,9 @@
       <c r="AN16" s="3"/>
       <c r="AO16" s="3"/>
       <c r="AP16" s="3"/>
-    </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ16" s="3"/>
+    </row>
+    <row r="17" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -7761,8 +7954,9 @@
       <c r="AN17" s="3"/>
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
-    </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ17" s="3"/>
+    </row>
+    <row r="18" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -7807,8 +8001,9 @@
       <c r="AN18" s="3"/>
       <c r="AO18" s="3"/>
       <c r="AP18" s="3"/>
-    </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ18" s="3"/>
+    </row>
+    <row r="19" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -7853,8 +8048,9 @@
       <c r="AN19" s="3"/>
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
-    </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ19" s="3"/>
+    </row>
+    <row r="20" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -7899,8 +8095,9 @@
       <c r="AN20" s="3"/>
       <c r="AO20" s="3"/>
       <c r="AP20" s="3"/>
-    </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ20" s="3"/>
+    </row>
+    <row r="21" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -7945,8 +8142,9 @@
       <c r="AN21" s="3"/>
       <c r="AO21" s="3"/>
       <c r="AP21" s="3"/>
-    </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ21" s="3"/>
+    </row>
+    <row r="22" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -7991,8 +8189,9 @@
       <c r="AN22" s="3"/>
       <c r="AO22" s="3"/>
       <c r="AP22" s="3"/>
-    </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ22" s="3"/>
+    </row>
+    <row r="23" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -8037,8 +8236,9 @@
       <c r="AN23" s="3"/>
       <c r="AO23" s="3"/>
       <c r="AP23" s="3"/>
-    </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ23" s="3"/>
+    </row>
+    <row r="24" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -8083,8 +8283,9 @@
       <c r="AN24" s="3"/>
       <c r="AO24" s="3"/>
       <c r="AP24" s="3"/>
-    </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ24" s="3"/>
+    </row>
+    <row r="25" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -8129,8 +8330,9 @@
       <c r="AN25" s="3"/>
       <c r="AO25" s="3"/>
       <c r="AP25" s="3"/>
-    </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ25" s="3"/>
+    </row>
+    <row r="26" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -8163,8 +8365,9 @@
       <c r="AN26" s="1"/>
       <c r="AO26" s="1"/>
       <c r="AP26" s="1"/>
-    </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ26" s="1"/>
+    </row>
+    <row r="27" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -8188,7 +8391,7 @@
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -8212,7 +8415,7 @@
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -8236,7 +8439,7 @@
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -8260,7 +8463,7 @@
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -8284,7 +8487,7 @@
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -8790,88 +8993,88 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="AG9:AP9"/>
+    <mergeCell ref="AG9:AQ9"/>
     <mergeCell ref="AA9:AF9"/>
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="34" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="7">
+    <cfRule type="expression" dxfId="35" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52 O11:R52">
-    <cfRule type="expression" dxfId="32" priority="19">
+    <cfRule type="expression" dxfId="34" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="31" priority="8">
+    <cfRule type="expression" dxfId="33" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="30" priority="9">
+    <cfRule type="expression" dxfId="32" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="29" priority="10">
+    <cfRule type="expression" dxfId="31" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="28" priority="13">
+    <cfRule type="expression" dxfId="30" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="27" priority="23">
+    <cfRule type="expression" dxfId="29" priority="23">
       <formula>$E11="cp"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="24">
+    <cfRule type="expression" dxfId="28" priority="24">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="25" priority="11">
+    <cfRule type="expression" dxfId="27" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="24" priority="12">
+    <cfRule type="expression" dxfId="26" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="23" priority="21">
+    <cfRule type="expression" dxfId="25" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="22" priority="14">
+    <cfRule type="expression" dxfId="24" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="21" priority="15">
+    <cfRule type="expression" dxfId="23" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="20" priority="16">
+    <cfRule type="expression" dxfId="22" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="19" priority="17">
+    <cfRule type="expression" dxfId="21" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="18" priority="1">
+  <conditionalFormatting sqref="AM11:AO52">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8918,183 +9121,183 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B2" s="3">
         <v>0.0</v>
       </c>
       <c r="D2" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="N2" s="24" t="s">
         <v>147</v>
-      </c>
-      <c r="N2" s="24" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B5" s="37">
         <v>1</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E5" s="37">
         <v>2</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="J5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K5" s="37">
         <v>4</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N5" s="37">
         <v>5</v>
       </c>
       <c r="P5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AC5" s="37">
         <v>10</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AR5" s="37">
         <v>15</v>
@@ -9187,172 +9390,172 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B7" s="37"/>
       <c r="D7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E7" s="37"/>
       <c r="G7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H7" s="37"/>
       <c r="J7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K7" s="37"/>
       <c r="M7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N7" s="37"/>
       <c r="P7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q7" s="37"/>
       <c r="R7" s="1"/>
       <c r="S7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T7" s="37"/>
       <c r="U7" s="1"/>
       <c r="V7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W7" s="37"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Z7" s="37"/>
       <c r="AA7" s="1"/>
       <c r="AB7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AC7" s="37"/>
       <c r="AE7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AF7" s="37"/>
       <c r="AG7" s="1"/>
       <c r="AH7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI7" s="37"/>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL7" s="37"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AO7" s="37"/>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR7" s="37"/>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="M8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="P8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="W8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="W8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="X8" s="1"/>
       <c r="Y8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Z8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AA8" s="1"/>
       <c r="AB8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="AC8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="AE8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AF8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AG8" s="1"/>
       <c r="AH8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AI8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AL8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AM8" s="1"/>
       <c r="AN8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AO8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AR8" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
@@ -10157,6 +10360,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -10173,20 +10390,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10220,10 +10423,10 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>168</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
@@ -10258,57 +10461,57 @@
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B5" s="39" t="inlineStr">
         <is>
@@ -10316,7 +10519,7 @@
         </is>
       </c>
       <c r="D5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E5" s="39" t="inlineStr">
         <is>
@@ -10324,7 +10527,7 @@
         </is>
       </c>
       <c r="G5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H5" s="39" t="inlineStr">
         <is>
@@ -10332,7 +10535,7 @@
         </is>
       </c>
       <c r="J5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K5" s="39" t="inlineStr">
         <is>
@@ -10340,7 +10543,7 @@
         </is>
       </c>
       <c r="M5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N5" s="39" t="inlineStr">
         <is>
@@ -10348,169 +10551,169 @@
         </is>
       </c>
       <c r="P5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="Q5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="T5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="T5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="W5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="W5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="Z5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="AC5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="AE5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AF5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AI5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AI5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AL5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AL5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AO5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AO5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AR5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AR5" s="39" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B6" s="39">
         <v>1</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E6" s="39">
         <v>2</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H6" s="39">
         <v>3</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K6" s="39">
         <v>3</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N6" s="39">
         <v>3</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q6" s="39">
         <v>6</v>
       </c>
       <c r="R6" s="1"/>
       <c r="S6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T6" s="39">
         <v>7</v>
       </c>
       <c r="U6" s="1"/>
       <c r="V6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="W6" s="39">
         <v>8</v>
       </c>
       <c r="X6" s="1"/>
       <c r="Y6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z6" s="39">
         <v>9</v>
       </c>
       <c r="AA6" s="1"/>
       <c r="AB6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AC6" s="39">
         <v>10</v>
       </c>
       <c r="AE6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AF6" s="39">
         <v>11</v>
       </c>
       <c r="AG6" s="1"/>
       <c r="AH6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AI6" s="39">
         <v>12</v>
       </c>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL6" s="39">
         <v>13</v>
       </c>
       <c r="AM6" s="1"/>
       <c r="AN6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO6" s="39">
         <v>14</v>
       </c>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AR6" s="39">
         <v>15</v>
@@ -10603,172 +10806,172 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B8" s="39"/>
       <c r="D8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E8" s="39"/>
       <c r="G8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H8" s="39"/>
       <c r="J8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K8" s="39"/>
       <c r="M8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N8" s="39"/>
       <c r="P8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q8" s="39"/>
       <c r="R8" s="1"/>
       <c r="S8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T8" s="39"/>
       <c r="U8" s="1"/>
       <c r="V8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W8" s="39"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Z8" s="39"/>
       <c r="AA8" s="1"/>
       <c r="AB8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AC8" s="39"/>
       <c r="AE8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AF8" s="39"/>
       <c r="AG8" s="1"/>
       <c r="AH8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI8" s="39"/>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL8" s="39"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AO8" s="39"/>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR8" s="39"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="M9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="P9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="W9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="X9" s="1"/>
       <c r="Y9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AA9" s="1"/>
       <c r="AB9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="AC9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="AE9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AF9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AG9" s="1"/>
       <c r="AH9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AI9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AJ9" s="1"/>
       <c r="AK9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AL9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AM9" s="1"/>
       <c r="AN9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AO9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AP9" s="1"/>
       <c r="AQ9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AR9" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
@@ -11669,6 +11872,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -11685,93 +11902,79 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>AND($B$5&lt;&gt;"",$B$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6 D7:E7">
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>AND($E$5&lt;&gt;"",$E$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 G7:H7">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>AND($H$5&lt;&gt;"",$H$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6 J7:K7">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>AND($K$5&lt;&gt;"",$K$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N6 M7:N7">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>AND($N$5&lt;&gt;"",$N$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q6 P7:Q7">
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>AND($Q$5&lt;&gt;"",$Q$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T6 S7:T7">
-    <cfRule type="expression" dxfId="11" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>AND($T$5&lt;&gt;"",$T$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W6 V7:W7">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="12" priority="8">
       <formula>AND($W$5&lt;&gt;"",$W$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z6 Y7:Z7">
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="11" priority="9">
       <formula>AND($Z$5&lt;&gt;"",$Z$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC6 AB7:AC7">
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="10" priority="10">
       <formula>AND($AC$5&lt;&gt;"",$AC$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6 AE7:AF7">
-    <cfRule type="expression" dxfId="7" priority="11">
+    <cfRule type="expression" dxfId="9" priority="11">
       <formula>AND($AF$5&lt;&gt;"",$AF$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI6 AH7:AI7">
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="8" priority="12">
       <formula>AND($AI$5&lt;&gt;"",$AI$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL6 AK7:AL7">
-    <cfRule type="expression" dxfId="5" priority="13">
+    <cfRule type="expression" dxfId="7" priority="13">
       <formula>AND($AL$5&lt;&gt;"",$AL$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO6 AN7:AO7">
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($AO$5&lt;&gt;"",$AO$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR6 AQ7:AR7">
-    <cfRule type="expression" dxfId="3" priority="15">
+    <cfRule type="expression" dxfId="5" priority="15">
       <formula>AND($AR$5&lt;&gt;"",$AR$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11795,20 +11998,20 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="59" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B2" s="54"/>
       <c r="D2" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E2" s="54"/>
       <c r="G2" s="22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B3" s="33" t="inlineStr">
         <is>
@@ -11816,7 +12019,7 @@
         </is>
       </c>
       <c r="D3" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E3" s="35" t="inlineStr">
         <is>
@@ -11827,19 +12030,19 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G4" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -11852,7 +12055,7 @@
         <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -11861,10 +12064,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H6" t="s">
         <v>192</v>
-      </c>
-      <c r="H6" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -12001,31 +12204,31 @@
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="D2" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="J2" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>5</v>
@@ -12053,10 +12256,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="J3" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -12071,10 +12274,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>204</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -12089,10 +12292,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K5" t="s">
         <v>206</v>
-      </c>
-      <c r="K5" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -12119,7 +12322,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="J7" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -12134,7 +12337,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K8"/>
     </row>
@@ -12150,7 +12353,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K9"/>
     </row>
@@ -12166,7 +12369,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="J10" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K10"/>
     </row>
@@ -12182,7 +12385,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K11"/>
     </row>
@@ -12198,31 +12401,31 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K12"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J13" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K13"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J14" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K14"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J15" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K15"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J16" s="14" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -12231,23 +12434,23 @@
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K17"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12272,16 +12475,16 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>221</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>5</v>
@@ -12292,10 +12495,10 @@
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F3" t="s">
         <v>222</v>
-      </c>
-      <c r="F3" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -12303,10 +12506,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="E4" t="s">
+        <v>223</v>
+      </c>
+      <c r="F4" t="s">
         <v>224</v>
-      </c>
-      <c r="F4" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -12314,10 +12517,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" t="s">
         <v>226</v>
-      </c>
-      <c r="F5" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -12447,122 +12650,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="61" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="61" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="61" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="61" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="61" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="61" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="P6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="X6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -12996,122 +13199,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="63" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="63" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="63" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="63" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="63" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="63" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="P6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="X6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">

</xml_diff>